<commit_message>
fix: refresh public instructions and bundle artifacts
</commit_message>
<xml_diff>
--- a/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
+++ b/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="Rcc0d7a640ac34455"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="Rb7eeabbee33e4405"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="R7d9b00dfaa1c4620"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="Rf8ffbbbfc2a74ae8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23918,7 +23918,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09a115a4396747db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra308b7105d124712"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: refresh immersive English scenes public package
</commit_message>
<xml_diff>
--- a/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
+++ b/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="R7d9b00dfaa1c4620"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="Rf8ffbbbfc2a74ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="Rb0900c14df894f65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R762d6e577dc4457f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23918,7 +23918,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra308b7105d124712"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf99658b4702342e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: tighten manga handoff contract and rebuild public bundle
</commit_message>
<xml_diff>
--- a/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
+++ b/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="Rb0900c14df894f65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R762d6e577dc4457f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="R500bb540d0e0405e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R286b1d28466240b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23918,7 +23918,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf99658b4702342e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84f1865e47594084"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: enforce explicit image tool completion semantics for manga flow
</commit_message>
<xml_diff>
--- a/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
+++ b/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="R500bb540d0e0405e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R286b1d28466240b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="R2e47a196c90c4a20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="Rf143f9193aef4843"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23918,7 +23918,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84f1865e47594084"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc43678451f0f4863"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: enforce manga image prompt format and prompt-block guards
</commit_message>
<xml_diff>
--- a/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
+++ b/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="R2e47a196c90c4a20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="Rf143f9193aef4843"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="R9693a2ba35264fbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="Rd38c9ad120794ec6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23918,7 +23918,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc43678451f0f4863"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c42f1768b0240aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: guard scene handoff from image-tool misrouting
</commit_message>
<xml_diff>
--- a/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
+++ b/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="R9693a2ba35264fbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="Rd38c9ad120794ec6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="Rd8be25f68b58402f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R126cf516f62346f1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23918,7 +23918,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c42f1768b0240aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad50a5ac6d6d46d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: strengthen image-tool argument guard for final-document misrouting
</commit_message>
<xml_diff>
--- a/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
+++ b/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="Rd8be25f68b58402f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R126cf516f62346f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="Rf382b2c26a9f4a86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R7ae03684a1494c7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23918,7 +23918,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad50a5ac6d6d46d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R706323598c8f424a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: materialize post-scene image guards in public artifacts
</commit_message>
<xml_diff>
--- a/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
+++ b/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="Rf382b2c26a9f4a86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R7ae03684a1494c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="Ra0034ce100e74c63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R448f38b6ad244096"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23918,7 +23918,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R706323598c8f424a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8324b8b3d12f4b53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: tighten post-scene image gate and roleplay firewall
</commit_message>
<xml_diff>
--- a/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
+++ b/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="Ra0034ce100e74c63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R448f38b6ad244096"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="R18d66512d2e949d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="Rfd1d1d5033c64b20"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23918,7 +23918,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8324b8b3d12f4b53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30fc2bef3f6f4066"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: replace enumerated image-block phrases with a generic scene state machine
A live E2E test proved the previous approach (enumerating specific
phrases like "Please send the final document" as roleplay-only)
insufficient: the model still fired the image tool for a request that
matched that exact list, producing a standalone document image before
review/handoff instead of the manga.

Replace it with a categorical gate: ROLEPLAY, CLOSING, REVIEW, and
HANDOFF are unconditionally text-only regardless of learner wording;
MANGA is entered only once REVIEW and HANDOFF are both visibly
complete, and allows exactly one image-tool call for the retrospective
manga — never the object the learner asked for. Also removes three
empty section-header stubs (ROLEPLAY TOOL FIREWALL / POST-SCENE IMAGE
GATE / MANGA-ONLY IMAGE RULE) that shipped with no body text.
</commit_message>
<xml_diff>
--- a/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
+++ b/UPLOAD_THESE_5_FILES/IES_v8_01_SCENE_CATALOG.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="R18d66512d2e949d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="Rfd1d1d5033c64b20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Start" sheetId="1" r:id="Rfeb732cdd09949e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Catalog" sheetId="2" r:id="R21a824c1e61346fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23918,7 +23918,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30fc2bef3f6f4066"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cdaa1a378654a32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>